<commit_message>
Mise à jour des entrées CDA (#120) 196f169c4ba76293996d90e2791aeb28e1d76d3e
</commit_message>
<xml_diff>
--- a/fusionEntreesCDA/ig/StructureDefinition-fr-cda-item-plan-traitement.xlsx
+++ b/fusionEntreesCDA/ig/StructureDefinition-fr-cda-item-plan-traitement.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-17T09:38:40+00:00</t>
+    <t>2026-04-20T06:44:24+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -6037,7 +6037,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="38" hidden="true">
+    <row r="38">
       <c r="A38" t="s" s="2">
         <v>175</v>
       </c>
@@ -6056,7 +6056,7 @@
         <v>75</v>
       </c>
       <c r="H38" t="s" s="2">
-        <v>74</v>
+        <v>169</v>
       </c>
       <c r="I38" t="s" s="2">
         <v>74</v>
@@ -6342,7 +6342,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="41" hidden="true">
+    <row r="41">
       <c r="A41" t="s" s="2">
         <v>183</v>
       </c>
@@ -6357,13 +6357,13 @@
         <v>62</v>
       </c>
       <c r="F41" t="s" s="2">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G41" t="s" s="2">
         <v>75</v>
       </c>
       <c r="H41" t="s" s="2">
-        <v>74</v>
+        <v>169</v>
       </c>
       <c r="I41" t="s" s="2">
         <v>74</v>
@@ -6445,7 +6445,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="42" hidden="true">
+    <row r="42">
       <c r="A42" t="s" s="2">
         <v>187</v>
       </c>
@@ -6460,13 +6460,13 @@
         <v>188</v>
       </c>
       <c r="F42" t="s" s="2">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G42" t="s" s="2">
         <v>75</v>
       </c>
       <c r="H42" t="s" s="2">
-        <v>74</v>
+        <v>169</v>
       </c>
       <c r="I42" t="s" s="2">
         <v>74</v>
@@ -6754,7 +6754,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="45" hidden="true">
+    <row r="45">
       <c r="A45" t="s" s="2">
         <v>201</v>
       </c>
@@ -6769,13 +6769,13 @@
         <v>202</v>
       </c>
       <c r="F45" t="s" s="2">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G45" t="s" s="2">
         <v>75</v>
       </c>
       <c r="H45" t="s" s="2">
-        <v>74</v>
+        <v>169</v>
       </c>
       <c r="I45" t="s" s="2">
         <v>74</v>

</xml_diff>